<commit_message>
Updated statistical tests and corresponding data and figures
</commit_message>
<xml_diff>
--- a/manu_sourcedata/extended_data_fig8.xlsx
+++ b/manu_sourcedata/extended_data_fig8.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yyj/Doc/1_dod_dec25/manu_sourcedata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA3E9AB8-4B61-FC43-8E96-6313D41D9EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CA0C15-6F7D-B442-B94A-5F59AE406711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{ED1ECD1F-5193-4245-9D87-00687259A86C}"/>
+    <workbookView xWindow="10080" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{ED1ECD1F-5193-4245-9D87-00687259A86C}"/>
   </bookViews>
   <sheets>
-    <sheet name="7a" sheetId="1" r:id="rId1"/>
+    <sheet name="8a" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>

</xml_diff>